<commit_message>
Kap 13 + ordbog
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gentoftehf-my.sharepoint.com/personal/hv_ghf_dk/Documents/GHF2/kemibog/kemic-web-2026/henryvest70.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{BCA33B2C-D84F-4566-A23B-2D2B12BCD0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A3EBA65-9A79-4CBF-959F-42F960362A9B}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{BCA33B2C-D84F-4566-A23B-2D2B12BCD0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EE7915D-9CCF-4DC7-89F5-40F5EA652D0C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AEC7298E-8AB4-4483-8A56-F40812FF3C99}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>forside</t>
   </si>
@@ -120,6 +120,12 @@
   </si>
   <si>
     <t>kemi b</t>
+  </si>
+  <si>
+    <t>kernebeg.</t>
+  </si>
+  <si>
+    <t>korr. Til 14.3</t>
   </si>
 </sst>
 </file>
@@ -551,6 +557,7 @@
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
       <c r="F1" s="2" t="s">
         <v>20</v>
       </c>
@@ -563,6 +570,9 @@
       <c r="C2" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="D2" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="F2" t="s">
         <v>21</v>
       </c>
@@ -580,11 +590,14 @@
       <c r="C3" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="D3" s="1" t="b">
+        <v>1</v>
+      </c>
       <c r="F3" t="s">
         <v>22</v>
       </c>
       <c r="G3" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -595,6 +608,9 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="b">
         <v>1</v>
       </c>
       <c r="F4" t="s">
@@ -614,6 +630,9 @@
       <c r="C5" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="D5" s="1" t="b">
+        <v>1</v>
+      </c>
       <c r="F5" t="s">
         <v>24</v>
       </c>
@@ -631,6 +650,9 @@
       <c r="C6" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="D6" s="1" t="b">
+        <v>1</v>
+      </c>
       <c r="F6" t="s">
         <v>18</v>
       </c>
@@ -648,6 +670,9 @@
       <c r="C7" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="D7" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -659,6 +684,9 @@
       <c r="C8" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="D8" s="1" t="b">
+        <v>1</v>
+      </c>
       <c r="F8" s="3" t="s">
         <v>25</v>
       </c>
@@ -671,7 +699,10 @@
         <v>1</v>
       </c>
       <c r="C9" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="F9" t="s">
         <v>26</v>
@@ -688,7 +719,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -699,7 +733,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -710,7 +747,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -721,7 +761,10 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -732,7 +775,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D14" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -743,7 +789,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -754,10 +803,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -767,8 +819,14 @@
       <c r="C17" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -776,10 +834,13 @@
         <v>1</v>
       </c>
       <c r="C18" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -787,7 +848,10 @@
         <v>1</v>
       </c>
       <c r="C19" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D19" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>